<commit_message>
Limpeza facial: conteúdo total no fim do descritivo dos kits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/LIMPEZA_FACIAL_descritivo.xlsx
+++ b/LIMPEZA_FACIAL_descritivo.xlsx
@@ -1813,7 +1813,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>KIT CENTELLA AMPOLA 125ML + OLEO DE LIMPEZA 200ML</t>
+          <t>KIT CENTELLA AMPOLA 125ML + OLEO DE LIMPEZA 200ML 325ML</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>KIT GARNIER SERUM 100G + HIDRATANTE 85G</t>
+          <t>KIT GARNIER SERUM 100G + HIDRATANTE 85G 180G</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>KIT LOREAL AGUA MICELAR 1.2L + PROTETOR SOLAR 25G</t>
+          <t>KIT LOREAL AGUA MICELAR 1.2L + PROTETOR SOLAR 25G 1.225L</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>KIT LOREAL REVITALIFT HIALURONICO 49G + GEL 80G + SERUM</t>
+          <t>KIT LOREAL REVITALIFT HIALURONICO 49G + GEL 80G + SERUM 129G</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>KIT DERMACHEM SABONETE 100ML + ESFOLIANTE 100ML</t>
+          <t>KIT DERMACHEM SABONETE 100ML + ESFOLIANTE 100ML 200ML</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>KIT DERMACHEM ESFOLIANTE 100G + SABONETE 100ML</t>
+          <t>KIT DERMACHEM ESFOLIANTE 100G + SABONETE 100ML 200ML</t>
         </is>
       </c>
     </row>
@@ -3490,7 +3490,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>KIT DERMACHEM VITAMINA C ESFOLIANTE 100G + SABONETE 100ML</t>
+          <t>KIT DERMACHEM ESFOLIANTE 100G + SABONETE 100ML 200ML</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>KIT ZETA SKIN SABONETE 300ML + SERUM 30ML</t>
+          <t>KIT ZETA SKIN SABONETE 300ML + SERUM 30ML 330ML</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>KIT ZETA SKIN SABONETE 300ML + SERUM 30ML</t>
+          <t>KIT ZETA SKIN SABONETE 300ML + SERUM 30ML 330ML</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>KIT LOREAL SERUM 30ML + CREME DIURNO 49G + CREME OLHOS 15G</t>
+          <t>KIT LOREAL SERUM 30ML + DIURNO 49G + CREME OLHOS 15G 94G</t>
         </is>
       </c>
     </row>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>OLEO DE LIMPEZA HADA LABO 200ML + REFIL 180ML</t>
+          <t>OLEO DE LIMPEZA HADA LABO 200ML + REFIL 180ML 380ML</t>
         </is>
       </c>
     </row>
@@ -5791,7 +5791,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>KIT HADA LABO OLEO 200ML + ESCOVA 1UN</t>
+          <t>KIT HADA LABO OLEO 200ML + ESCOVA 1UN 200ML</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HIDRATANTE 30G</t>
+          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HID 30G 150ML</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HIDRATANTE 30G</t>
+          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HID 30G 150ML</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6844,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>KIT NUPILL FIRMNESS SABONETE 60ML + LOCAO 60ML + GEL 50ML</t>
+          <t>KIT NUPILL SABONETE 60ML + LOCAO 60ML + GEL 50ML 170ML</t>
         </is>
       </c>
     </row>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HIDRATANTE 30G</t>
+          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HID 30G 150ML</t>
         </is>
       </c>
     </row>
@@ -7312,7 +7312,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HIDRATANTE 30G</t>
+          <t>KIT NUPILL SABONETE 60ML + TONICO 60ML + HID 30G 150ML</t>
         </is>
       </c>
     </row>
@@ -8131,7 +8131,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>KIT DAUF PROTETOR SOLAR 35ML + HIDRATANTE 35G + SABONETE 35G</t>
+          <t>KIT DAUF PROTETOR SOLAR 35ML + HID 35G + SABONETE 35G 3UN</t>
         </is>
       </c>
     </row>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>KIT LABOTRAT SAB 100ML + AGUA MICELAR 110ML + SERUM 30ML</t>
+          <t>KIT LABOTRAT SAB 100ML + MICELAR 110ML + SERUM 30ML 240ML</t>
         </is>
       </c>
     </row>
@@ -9535,7 +9535,7 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>KIT LABOTRAT SABONETE 100ML + TONICO 100ML + GEL 15G</t>
+          <t>KIT LABOTRAT SABONETE 100ML + TONICO 100ML + GEL 15G 230ML</t>
         </is>
       </c>
     </row>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>KIT LABOTRAT SABONETE 100ML + TONICO 100ML + GEL 15G</t>
+          <t>KIT LABOTRAT SABONETE 100ML + TONICO 100ML + GEL 15G 215ML</t>
         </is>
       </c>
     </row>
@@ -10315,7 +10315,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>KIT GLANCE CARE DEMAQ 60ML + SABONETE 60ML + ESFOLIANTE 60ML</t>
+          <t>KIT GLANCE CARE DEMAQ 60ML + SAB 60ML + ESFOL 60ML 180ML</t>
         </is>
       </c>
     </row>
@@ -11329,7 +11329,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>KIT DAXX SABONETE + LENCO UMEDECIDO</t>
+          <t>KIT DAXX SABONETE + LENCO UMEDECIDO 250ML</t>
         </is>
       </c>
     </row>
@@ -11368,7 +11368,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>KIT DAXX SABONETE + LENCO UMEDECIDO</t>
+          <t>KIT DAXX SABONETE + LENCO UMEDECIDO 1L</t>
         </is>
       </c>
     </row>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>KIT VINI LADY SABONETE 95ML + TONICO 150ML</t>
+          <t>KIT VINI LADY SABONETE 95ML + TONICO 150ML 245ML</t>
         </is>
       </c>
     </row>
@@ -12070,7 +12070,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>KIT VINI LADY CONTROLE BRILHO SABONETE 95ML + TONICO 150ML</t>
+          <t>KIT VINI LADY SABONETE 95ML + TONICO 150ML 245ML</t>
         </is>
       </c>
     </row>
@@ -12148,7 +12148,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>KIT FOR MEN ESPUMA + GEL</t>
+          <t>KIT FOR MEN ESPUMA + GEL 150ML</t>
         </is>
       </c>
     </row>
@@ -12187,7 +12187,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>KIT ACNEZIL SABONETE 200ML + PROTETOR SOLAR 60G + GEL 10G</t>
+          <t>KIT ACNEZIL SAB 200ML + PROTETOR SOLAR 60G + GEL 10G 530ML</t>
         </is>
       </c>
     </row>
@@ -12226,7 +12226,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>KIT ACNEZIL SABONETE 200ML + LOCAO 200ML + GEL 10G</t>
+          <t>KIT ACNEZIL SABONETE 200ML + LOCAO 200ML + GEL 10G 410ML</t>
         </is>
       </c>
     </row>
@@ -12343,7 +12343,7 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>KIT GALDERMA HIDRATANTE 50ML + SABONETE 70ML</t>
+          <t>KIT GALDERMA HIDRATANTE 50ML + SABONETE 70ML 120ML</t>
         </is>
       </c>
     </row>
@@ -13474,7 +13474,7 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>KIT HIDRAMAIS GEL 110ML + FLUIDO 120ML + SECATIVO 20G</t>
+          <t>KIT HIDRAMAIS GEL 110ML + FLUIDO 120ML + SECATIVO 20G 250ML</t>
         </is>
       </c>
     </row>
@@ -13513,7 +13513,7 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>KIT HIDRAMAIS FLUIDO 120ML + MASCARA 50G + HIDRATANTE 50G</t>
+          <t>KIT HIDRAMAIS FLUIDO 120ML + MASCARA 50G + HID 50G 220ML</t>
         </is>
       </c>
     </row>
@@ -16828,7 +16828,7 @@
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>KIT SIMPLE HIDRATANTE 50ML + SABONETE 50ML + LENCO 7UN</t>
+          <t>KIT SIMPLE HIDRATANTE 50ML + SABONETE 50ML + LENCO 7UN 107ML</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Limpeza facial: tipo do item no início do descritivo (OUTRO LIMPEZA FACIAL)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/LIMPEZA_FACIAL_descritivo.xlsx
+++ b/LIMPEZA_FACIAL_descritivo.xlsx
@@ -1462,7 +1462,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA ROSA 24X200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA ROSA 24X200ML</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TOQUE CARINHO 12X200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TOQUE CARINHO 12X200ML</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TOQUE CARINHO 12X200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TOQUE CARINHO 12X200ML</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TEMPO AMAR 12X200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TEMPO AMAR 12X200ML</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA ORIGINAL 12X200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA ORIGINAL 12X200ML</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3529,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>ADSTRINGENTE FACIAL DERMACHEM ADSTRIGENTE 120ML</t>
+          <t>ADSTRINGENTE FACIAL DERMACHEM 120ML</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL B O BARRA PELE OLEOSA 55G</t>
+          <t>BARRA DE LIMPEZA B O PELE OLEOSA 55G</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL B O BARRA PELE NORMAL 90G</t>
+          <t>BARRA DE LIMPEZA B O PELE NORMAL 90G</t>
         </is>
       </c>
     </row>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL CAPIM LIMAO SACHE BLACK MASK REMOVEDOR 8G</t>
+          <t>MASCARA FACIAL CAPIM LIMAO SACHE BLACK MASK REMOVEDOR 8G</t>
         </is>
       </c>
     </row>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>ESFOLIANTE FACIAL KIND BEAUTY POLPA SUAVE MARACUJA 80G</t>
+          <t>POLPA DE LIMPEZA KIND BEAUTY ESFOLIANTE SUAVE MARACUJA 80G</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL KIND BEAUTY POLPA DETOX 80G</t>
+          <t>POLPA DE LIMPEZA KIND BEAUTY FACIAL DETOX 80G</t>
         </is>
       </c>
     </row>
@@ -10081,7 +10081,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL NINA MAKE UP SABOENTE HYALURONIC CARE 120ML</t>
+          <t>SABONETE FACIAL NINA MAKE UP HYALURONIC CARE 120ML</t>
         </is>
       </c>
     </row>
@@ -11446,7 +11446,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL NATUFLORES LEITE ROSA MOSQUETA 120ML</t>
+          <t>LEITE DE LIMPEZA FACIAL NATUFLORES ROSA MOSQUETA 120ML</t>
         </is>
       </c>
     </row>
@@ -12577,7 +12577,7 @@
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL HIDRABENE ESMPUMA 100ML</t>
+          <t>ESPUMA FACIAL HIDRABENE 100ML</t>
         </is>
       </c>
     </row>
@@ -14683,7 +14683,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TOQUE CARINHO 200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TOQUE CARINHO 200ML</t>
         </is>
       </c>
     </row>
@@ -14722,7 +14722,7 @@
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TOQUE CARINHO 100ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TOQUE CARINHO 100ML</t>
         </is>
       </c>
     </row>
@@ -14761,7 +14761,7 @@
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TEMPO AMAR 200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TEMPO AMAR 200ML</t>
         </is>
       </c>
     </row>
@@ -14800,7 +14800,7 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA TEMPO AMAR 100ML</t>
+          <t>DESODORANTE LEITE DE COLONIA TEMPO AMAR 100ML</t>
         </is>
       </c>
     </row>
@@ -14839,7 +14839,7 @@
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA FINAL FANTASTIC 200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA FINAL FANTASTIC 200ML</t>
         </is>
       </c>
     </row>
@@ -14917,7 +14917,7 @@
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA ORIGINAL 200ML</t>
+          <t>DESODORANTE LEITE DE COLONIA ORIGINAL 200ML</t>
         </is>
       </c>
     </row>
@@ -14956,7 +14956,7 @@
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL LEITE DE COLONIA ORIGINAL 100ML</t>
+          <t>DESODORANTE LEITE DE COLONIA ORIGINAL 100ML</t>
         </is>
       </c>
     </row>
@@ -16321,7 +16321,7 @@
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL DAILUS CLEASING BALM SWEET SKIN 100G</t>
+          <t>BALM DE LIMPEZA DAILUS SWEET SKIN 100G</t>
         </is>
       </c>
     </row>
@@ -16438,7 +16438,7 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL PULSY POMADA LIMPA PELE 30G</t>
+          <t>POMADA FACIAL PULSY LIMPA PELE 30G</t>
         </is>
       </c>
     </row>
@@ -17374,7 +17374,7 @@
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t>LIMPEZA FACIAL CLEAN CLEAR CC ADSTRING PROFUNDA 200ML</t>
+          <t>ADSTRINGENTE FACIAL CLEAN CLEAR CC PROFUNDA 200ML</t>
         </is>
       </c>
     </row>
@@ -18739,7 +18739,7 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>OLEO DE LIMPEZA KISS NEW YORK FACIAL YOUNG CLEANSING 80G</t>
+          <t>BALM DE LIMPEZA KISS NEW YORK YOUNG 80G</t>
         </is>
       </c>
     </row>

</xml_diff>